<commit_message>
version 43 - Update Design + REST API
</commit_message>
<xml_diff>
--- a/Documentation/API/RESTFul_API.xlsx
+++ b/Documentation/API/RESTFul_API.xlsx
@@ -176,7 +176,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="233">
   <si>
     <t>RESTfull API</t>
   </si>
@@ -661,6 +661,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
       <t>+ If user is valid:</t>
     </r>
     <r>
@@ -862,10 +868,7 @@
     <t>/api/Add_new_product</t>
   </si>
   <si>
-    <t>Waiting to implement with admin</t>
-  </si>
-  <si>
-    <t>ADD_NEW_PRODUCT_URL</t>
+    <t>Delicated (covered by Candle Add New Product)</t>
   </si>
   <si>
     <t>API 17: Payment handling</t>
@@ -1000,6 +1003,482 @@
   </si>
   <si>
     <t>All internal Angular routing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">API 20: </t>
+  </si>
+  <si>
+    <t>MySQL_TestConnection</t>
+  </si>
+  <si>
+    <t>/api/mysql</t>
+  </si>
+  <si>
+    <t>/</t>
+  </si>
+  <si>
+    <t>For testing</t>
+  </si>
+  <si>
+    <t>API 21: Get Data from MongoDB and merge with MySQL Warehouse</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>/api/admin/update_warehouse_mysql</t>
+  </si>
+  <si>
+    <t>API 22: Payment PayPal gateway</t>
+  </si>
+  <si>
+    <t>Payment_Paypal</t>
+  </si>
+  <si>
+    <t>/api/payment/paypal</t>
+  </si>
+  <si>
+    <t>/show_detail</t>
+  </si>
+  <si>
+    <t>Frontend call to Backend , Backend call to PayPal API to get detail of order based on Order ID</t>
+  </si>
+  <si>
+    <t>'- OrderID
+- Access Token valid</t>
+  </si>
+  <si>
+    <t>Format output will follow with PayPal API</t>
+  </si>
+  <si>
+    <t>Not implement - Will plan</t>
+  </si>
+  <si>
+    <t>/create-order</t>
+  </si>
+  <si>
+    <t>Frontend call to Backend and Backend will call to PayPal API for create Order</t>
+  </si>
+  <si>
+    <t>{
+    Selected_List_Object?: Array&lt;Selected_Candle&gt;;
+    Price_currency?:string;
+}
+AND
+Access Token valid</t>
+  </si>
+  <si>
+    <t>Return Order ID from PayPal</t>
+  </si>
+  <si>
+    <t>Create_Order_URL</t>
+  </si>
+  <si>
+    <t>/capture-order</t>
+  </si>
+  <si>
+    <t>After User paid sucessfully, Frontend will call to Backend, Backend call to PayPal API to confirm order based on Order ID</t>
+  </si>
+  <si>
+    <t>Capture_Order_URL</t>
+  </si>
+  <si>
+    <t>API 23: Payment VNPay gateway</t>
+  </si>
+  <si>
+    <t>Payment_VNPay</t>
+  </si>
+  <si>
+    <t>/api/payment/vnpay</t>
+  </si>
+  <si>
+    <t>/create_payment_url</t>
+  </si>
+  <si>
+    <t>Frontend send request to Backend to create Official URL to VNPay based on needed information. Backend will generate final URL in this route and send to Frontend (Frontend will open URL)</t>
+  </si>
+  <si>
+    <t>{
+    amount_for_VNPay?:string;
+    bankCode_for_VNPay?:string;
+    language_for_VNPay?:string;
+  }
+AND
+TmnCode &amp; HashSecret valid</t>
+  </si>
+  <si>
+    <t>{
+    vnpUrl,
+    orderId
+}</t>
+  </si>
+  <si>
+    <t>Create_VNPAY_Order_URL</t>
+  </si>
+  <si>
+    <t>/vnpay_return</t>
+  </si>
+  <si>
+    <t>Browser will call this URL to Backend after have result of payment</t>
+  </si>
+  <si>
+    <t>req.query
+AND
+TmnCode &amp; HashSecret valid</t>
+  </si>
+  <si>
+    <r>
+      <t>If Signature is Valid</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">
+{
+       status_order_vnpay_return = 'PAID_With_VNPay_Return';
+        res.status(200).send(
+        [{
+            "VNPay_Result" : "success",
+            "code" : `${vnp_Params['vnp_ResponseCode']}`
+        }])
+    } 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t>else if Signature is Invalid</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">
+{
+       status_order_vnpay_return = 'FAILED_With_VNPay_Return';
+        res.status(200).send(
+        [{
+            "VNPay_Result" : "success",
+            "code" : '97'
+        }])
+    }</t>
+    </r>
+  </si>
+  <si>
+    <t>N/A (User browset auto redirect)</t>
+  </si>
+  <si>
+    <t>/vnpay_ipn</t>
+  </si>
+  <si>
+    <t>VNPay Server will call to Backend, for inform official payment result (Only applicable for Production)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">If Signature is Valid &amp; Payment sucessfully:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">status_order_vnpay_ipn = 'PAID_PAYMENT_With_VNPay_IPN';
+res.status(200).json({RspCode: '00', Message: 'Success'})
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t>If Signature is Valid &amp; Payment failed:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">
+status_order_vnpay_ipn = 'FAILED_PAYMENT_With_VNPay_IPN';
+res.status(200).json({RspCode: `${rspCode}`, Message: 'Failed'})
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t>If Signature is Valid &amp; Payment is checked before (avoid duplicate checking):</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">
+status_order_vnpay_ipn = 'HAS_DONE_UPDATED_VNPay_IPN';
+res.status(200).json({RspCode: `02`, Message: 'This order has been updated to the payment status'})
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t>If Signature is Valid &amp; Inconsistency amout money with Backend Database:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">
+status_order_vnpay_ipn = 'INCONSISTENCY_AMOUNT_VNPay_IPN';
+res.status(200).json({RspCode: `04`, Message: 'Amount invalid'})
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t>If Signature is Valid &amp; Inconsistency Order ID with Backend Database:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">
+status_order_vnpay_ipn = 'INCONSISTENCY_ORDER_VNPay_IPN';
+res.status(200).json({RspCode: `01`, Message: 'Order not found'})
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">
+If Signature is Invalid:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">
+status_order_vnpay_ipn = 'INCONSISTENCY_HASH_VNPay_IPN';
+res.status(200).json({RspCode: `97`, Message: 'Checksum failed'})
+</t>
+    </r>
+  </si>
+  <si>
+    <t>/querydr</t>
+  </si>
+  <si>
+    <t>Frontend will call to Backend many time to request confirm payment status both VNPAY_RETURN and VNPAY_IPN</t>
+  </si>
+  <si>
+    <t>req.query.orderId</t>
+  </si>
+  <si>
+    <t>{
+   status_order_vnpay_return,
+   status_order_vnpay_ipn,
+   req.query.orderId
+}</t>
+  </si>
+  <si>
+    <t>Check_status_Order_VNPay</t>
+  </si>
+  <si>
+    <t>API 24: Admin management gateway</t>
+  </si>
+  <si>
+    <t>Admin_management</t>
+  </si>
+  <si>
+    <t>/api/admin_management</t>
+  </si>
+  <si>
+    <t>/customer</t>
+  </si>
+  <si>
+    <t>Get all information about customer and display for admin right</t>
+  </si>
+  <si>
+    <t>Array of Object
+{
+         "Customer_Id" : `${customer.customer_id}`,
+         "email" : `${customer.email}`,
+         "name" : `${customer.name}`,
+         "address" : `${customer.address}`
+}</t>
+  </si>
+  <si>
+    <t>ADMIN_Customer_URL</t>
+  </si>
+  <si>
+    <t>/coupon</t>
+  </si>
+  <si>
+    <t>Get all information about coupon and display for admin right</t>
+  </si>
+  <si>
+    <t>Array of Object
+{
+         "Coupon_id" : `${coupon.coupon_id}`,
+         "Code" : `${coupon.code}`,
+         "Discount_type" : `${coupon.discount_type}`,
+         "Discount_value" : `${coupon.discount_value}`,
+         "MinOrderValue" : `${coupon.min_order_value}`,
+         "MaxDiscountValue" : `${coupon.max_discount_value}`,
+         "ValidFrom" : `${coupon.valid_from}`,
+         "ValidTo" : `${coupon.valid_to}`,
+         "UsageLimit" : `${coupon.usage_limit}`,
+         "LimitForPerson" : `${coupon.per_user_limit}`,
+         "StatusActivation" : `${coupon.status}`
+}</t>
+  </si>
+  <si>
+    <t>Update coupon status by admin right</t>
+  </si>
+  <si>
+    <t>Array of Object (that need  to be changed)
+{
+    coupon.Coupon_id,
+    coupon.StatusActivation
+}</t>
+  </si>
+  <si>
+    <t>{message: 'Coupon status updated successfully'}</t>
+  </si>
+  <si>
+    <t>ADMIN_Coupon_URL</t>
+  </si>
+  <si>
+    <t>/inventory</t>
+  </si>
+  <si>
+    <t>Get all information about inventory and display for admin right</t>
+  </si>
+  <si>
+    <t>Array of Object
+{
+         "InventoryId" : `${inventory.inventory_id}`,
+         "ProductName" : `${inventory.product_sku}`,
+         "Quantity" : `${inventory.quantity}`,
+         "WarehouseName" : `${inventory.name}`,
+         "Location" : `${inventory.location}`
+}</t>
+  </si>
+  <si>
+    <t>ADMIN_Inventory_URL</t>
+  </si>
+  <si>
+    <t>/warehouse</t>
+  </si>
+  <si>
+    <t>Get all information about warehouse and display for admin right</t>
+  </si>
+  <si>
+    <t>Array of Object
+{
+         "Warehouse_ID" : `${warehouse.warehouse_id }`,
+         "WarehouseName" : `${warehouse.name}`,
+         "Location" : `${warehouse.location}`,
+         "Capacity" : `${warehouse.capacity}`,
+         "ManagerName" : `${warehouse.manager_name}`
+}</t>
+  </si>
+  <si>
+    <t>ADMIN_Warehouse_URL</t>
+  </si>
+  <si>
+    <t>/orderstatus</t>
+  </si>
+  <si>
+    <t>Get all information about orderstatus and display for admin right</t>
+  </si>
+  <si>
+    <t>Array of Object
+{
+         "OrderId" : `${order_detail.order_id}`,
+         "CustomerId" : `${order_detail.customer_id}`,
+         "CustomerUsername" : `${order_detail.name}`,
+         "TotalAmount" : `${order_detail.total_amount}`,
+         "OrderStatus" : `${order_detail.status}`,
+         "OrderDate" : `${order_detail.order_date}`,
+         "details" : Array of Object
+                  {
+                      "OrderDetailId" : `${d.order_detail_id}`,
+                      "ProductName" : `${d.product_sku}`,
+                      "Quantity" : `${d.quantity}`,
+                      "UnitPrice" : `${d.unit_price}`,
+                      "SubTotalAmount" : `${d.subtotal}`,
+                      "PaymentId" : `${d.payment_id}`,
+                      "PaymentMethod" : `${d.method}`,
+                      "PaymentStatus" : `${d.status}`,
+                      "PaymentGatewayId" : `${d.payment_gateway_id}`
+                  }
+}</t>
+  </si>
+  <si>
+    <t>Update Order status by admin right</t>
+  </si>
+  <si>
+    <t>Array of Object (that need  to be changed)
+{
+    order.OrderId,
+    order.OrderStatus
+}</t>
+  </si>
+  <si>
+    <t>{message: 'Order status updated successfully'}</t>
+  </si>
+  <si>
+    <t>ADMIN_OrderStatus_URL</t>
   </si>
 </sst>
 </file>
@@ -1222,16 +1701,16 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-    </font>
-    <font>
       <b/>
       <i/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Arial"/>
       <charset val="134"/>
     </font>
     <font>
@@ -1246,7 +1725,7 @@
       <charset val="0"/>
     </font>
   </fonts>
-  <fills count="41">
+  <fills count="42">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1292,6 +1771,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2" tint="-0.25"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF808080"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1488,7 +1973,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -1497,7 +1982,37 @@
       <diagonal/>
     </border>
     <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
         <color auto="1"/>
       </left>
       <right style="thin">
@@ -1521,7 +2036,24 @@
       <top style="thin">
         <color auto="1"/>
       </top>
-      <bottom/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -1531,19 +2063,55 @@
       <right style="thin">
         <color auto="1"/>
       </right>
-      <top/>
-      <bottom/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
         <color auto="1"/>
       </left>
-      <right style="thin">
+      <right style="medium">
         <color auto="1"/>
       </right>
-      <top/>
+      <top style="medium">
+        <color auto="1"/>
+      </top>
       <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="medium">
         <color auto="1"/>
       </bottom>
       <diagonal/>
@@ -1670,7 +2238,7 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="10" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1682,119 +2250,119 @@
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="11" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="12" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="14" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="16" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="17" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="41" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1812,155 +2380,245 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2016,6 +2674,11 @@
     <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="00808080"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -2302,7 +2965,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:K33"/>
+  <dimension ref="A1:K47"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.4"/>
   <cols>
     <col min="1" max="1" width="38.5833333333333" style="2" customWidth="1"/>
@@ -2319,7 +2982,7 @@
     <col min="12" max="16384" width="9" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.8" spans="1:1">
+    <row r="1" ht="23.55" spans="1:1">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -2347,638 +3010,638 @@
       </c>
       <c r="I2" s="12"/>
       <c r="J2" s="12"/>
-      <c r="K2" s="45" t="s">
+      <c r="K2" s="63" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="3" s="1" customFormat="1" ht="23" customHeight="1" spans="1:11">
-      <c r="A3" s="6"/>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="13" t="s">
+      <c r="A3" s="13"/>
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="F3" s="13" t="s">
+      <c r="F3" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="G3" s="13" t="s">
+      <c r="G3" s="16" t="s">
         <v>10</v>
       </c>
-      <c r="H3" s="14" t="s">
+      <c r="H3" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="14" t="s">
+      <c r="I3" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="J3" s="14" t="s">
+      <c r="J3" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="K3" s="46"/>
+      <c r="K3" s="64"/>
     </row>
     <row r="4" s="2" customFormat="1" ht="54" customHeight="1" spans="1:11">
-      <c r="A4" s="15" t="s">
+      <c r="A4" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="17" t="s">
+      <c r="C4" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="18" t="s">
+      <c r="D4" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="50" t="s">
+      <c r="E4" s="79" t="s">
         <v>16</v>
       </c>
-      <c r="F4" s="19" t="s">
+      <c r="F4" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="G4" s="50" t="s">
+      <c r="G4" s="79" t="s">
         <v>18</v>
       </c>
-      <c r="H4" s="20" t="s">
+      <c r="H4" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="I4" s="25"/>
-      <c r="J4" s="25"/>
-      <c r="K4" s="51" t="s">
+      <c r="I4" s="26"/>
+      <c r="J4" s="26"/>
+      <c r="K4" s="80" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="5" s="1" customFormat="1" ht="147" customHeight="1" spans="1:11">
-      <c r="A5" s="21" t="s">
+      <c r="A5" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="B5" s="22" t="s">
+      <c r="B5" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="22" t="s">
+      <c r="C5" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="18" t="s">
+      <c r="D5" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="50" t="s">
+      <c r="E5" s="79" t="s">
         <v>24</v>
       </c>
-      <c r="F5" s="19" t="s">
+      <c r="F5" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="G5" s="50" t="s">
+      <c r="G5" s="79" t="s">
         <v>25</v>
       </c>
-      <c r="H5" s="20" t="s">
+      <c r="H5" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="I5" s="25"/>
-      <c r="J5" s="25"/>
-      <c r="K5" s="47" t="s">
+      <c r="I5" s="26"/>
+      <c r="J5" s="26"/>
+      <c r="K5" s="66" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="6" s="1" customFormat="1" ht="164" customHeight="1" spans="1:11">
-      <c r="A6" s="23"/>
-      <c r="B6" s="24"/>
-      <c r="C6" s="24"/>
-      <c r="D6" s="18" t="s">
+      <c r="A6" s="24"/>
+      <c r="B6" s="25"/>
+      <c r="C6" s="25"/>
+      <c r="D6" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="E6" s="20" t="s">
+      <c r="E6" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="F6" s="25"/>
-      <c r="G6" s="25"/>
-      <c r="H6" s="50" t="s">
+      <c r="F6" s="26"/>
+      <c r="G6" s="26"/>
+      <c r="H6" s="79" t="s">
         <v>28</v>
       </c>
-      <c r="I6" s="50" t="s">
+      <c r="I6" s="79" t="s">
         <v>29</v>
       </c>
-      <c r="J6" s="50" t="s">
+      <c r="J6" s="79" t="s">
         <v>30</v>
       </c>
-      <c r="K6" s="47" t="s">
+      <c r="K6" s="66" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="7" s="1" customFormat="1" ht="176.4" customHeight="1" spans="1:11">
-      <c r="A7" s="23"/>
-      <c r="B7" s="24"/>
-      <c r="C7" s="24"/>
-      <c r="D7" s="18" t="s">
+      <c r="A7" s="24"/>
+      <c r="B7" s="25"/>
+      <c r="C7" s="25"/>
+      <c r="D7" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="E7" s="52" t="s">
+      <c r="E7" s="81" t="s">
         <v>33</v>
       </c>
-      <c r="F7" s="26"/>
-      <c r="G7" s="26"/>
-      <c r="H7" s="20" t="s">
+      <c r="F7" s="27"/>
+      <c r="G7" s="27"/>
+      <c r="H7" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="I7" s="25"/>
-      <c r="J7" s="25"/>
-      <c r="K7" s="47" t="s">
+      <c r="I7" s="26"/>
+      <c r="J7" s="26"/>
+      <c r="K7" s="66" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="8" s="1" customFormat="1" ht="194" customHeight="1" spans="1:11">
-      <c r="A8" s="23"/>
-      <c r="B8" s="24"/>
-      <c r="C8" s="24"/>
-      <c r="D8" s="18" t="s">
+      <c r="A8" s="24"/>
+      <c r="B8" s="25"/>
+      <c r="C8" s="25"/>
+      <c r="D8" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="E8" s="20" t="s">
+      <c r="E8" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="F8" s="25"/>
-      <c r="G8" s="25"/>
-      <c r="H8" s="53" t="s">
+      <c r="F8" s="26"/>
+      <c r="G8" s="26"/>
+      <c r="H8" s="82" t="s">
         <v>36</v>
       </c>
-      <c r="I8" s="27" t="s">
+      <c r="I8" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="J8" s="27" t="s">
+      <c r="J8" s="28" t="s">
         <v>38</v>
       </c>
-      <c r="K8" s="36" t="s">
+      <c r="K8" s="67" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="9" s="1" customFormat="1" ht="194" customHeight="1" spans="1:11">
-      <c r="A9" s="28"/>
-      <c r="B9" s="29"/>
-      <c r="C9" s="29"/>
-      <c r="D9" s="18" t="s">
+      <c r="A9" s="24"/>
+      <c r="B9" s="25"/>
+      <c r="C9" s="25"/>
+      <c r="D9" s="21" t="s">
         <v>40</v>
       </c>
-      <c r="E9" s="20"/>
-      <c r="F9" s="25"/>
-      <c r="G9" s="25"/>
-      <c r="H9" s="53" t="s">
+      <c r="E9" s="23"/>
+      <c r="F9" s="26"/>
+      <c r="G9" s="26"/>
+      <c r="H9" s="82" t="s">
         <v>41</v>
       </c>
-      <c r="I9" s="27" t="s">
+      <c r="I9" s="28" t="s">
         <v>37</v>
       </c>
-      <c r="J9" s="27" t="s">
+      <c r="J9" s="28" t="s">
         <v>42</v>
       </c>
-      <c r="K9" s="36" t="s">
+      <c r="K9" s="67" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:11">
-      <c r="A10" s="30" t="s">
+      <c r="A10" s="29" t="s">
         <v>44</v>
       </c>
-      <c r="B10" s="25" t="s">
+      <c r="B10" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="C10" s="25" t="s">
+      <c r="C10" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="D10" s="31" t="s">
+      <c r="D10" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="E10" s="20" t="s">
+      <c r="E10" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="F10" s="25"/>
-      <c r="G10" s="25"/>
-      <c r="H10" s="20" t="s">
+      <c r="F10" s="26"/>
+      <c r="G10" s="26"/>
+      <c r="H10" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="I10" s="25"/>
-      <c r="J10" s="25"/>
-      <c r="K10" s="25" t="s">
+      <c r="I10" s="26"/>
+      <c r="J10" s="26"/>
+      <c r="K10" s="68" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="11" spans="1:11">
-      <c r="A11" s="30" t="s">
+      <c r="A11" s="29" t="s">
         <v>49</v>
       </c>
-      <c r="B11" s="25" t="s">
+      <c r="B11" s="26" t="s">
         <v>50</v>
       </c>
-      <c r="C11" s="25" t="s">
+      <c r="C11" s="26" t="s">
         <v>51</v>
       </c>
-      <c r="D11" s="31" t="s">
+      <c r="D11" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="E11" s="20" t="s">
+      <c r="E11" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="F11" s="25"/>
-      <c r="G11" s="25"/>
-      <c r="H11" s="20" t="s">
+      <c r="F11" s="26"/>
+      <c r="G11" s="26"/>
+      <c r="H11" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="I11" s="25"/>
-      <c r="J11" s="25"/>
-      <c r="K11" s="25" t="s">
+      <c r="I11" s="26"/>
+      <c r="J11" s="26"/>
+      <c r="K11" s="68" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:11">
-      <c r="A12" s="30" t="s">
+      <c r="A12" s="29" t="s">
         <v>53</v>
       </c>
-      <c r="B12" s="25" t="s">
+      <c r="B12" s="26" t="s">
         <v>54</v>
       </c>
-      <c r="C12" s="25" t="s">
+      <c r="C12" s="26" t="s">
         <v>55</v>
       </c>
-      <c r="D12" s="31" t="s">
+      <c r="D12" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="E12" s="20" t="s">
+      <c r="E12" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="F12" s="25"/>
-      <c r="G12" s="25"/>
-      <c r="H12" s="20" t="s">
+      <c r="F12" s="26"/>
+      <c r="G12" s="26"/>
+      <c r="H12" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="I12" s="25"/>
-      <c r="J12" s="25"/>
-      <c r="K12" s="25" t="s">
+      <c r="I12" s="26"/>
+      <c r="J12" s="26"/>
+      <c r="K12" s="68" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="30" t="s">
+      <c r="A13" s="29" t="s">
         <v>57</v>
       </c>
-      <c r="B13" s="25" t="s">
+      <c r="B13" s="26" t="s">
         <v>58</v>
       </c>
-      <c r="C13" s="25" t="s">
+      <c r="C13" s="26" t="s">
         <v>59</v>
       </c>
-      <c r="D13" s="31" t="s">
+      <c r="D13" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="E13" s="20" t="s">
+      <c r="E13" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="F13" s="25"/>
-      <c r="G13" s="25"/>
-      <c r="H13" s="20" t="s">
+      <c r="F13" s="26"/>
+      <c r="G13" s="26"/>
+      <c r="H13" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="I13" s="25"/>
-      <c r="J13" s="25"/>
-      <c r="K13" s="25" t="s">
+      <c r="I13" s="26"/>
+      <c r="J13" s="26"/>
+      <c r="K13" s="68" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="30" t="s">
+      <c r="A14" s="29" t="s">
         <v>61</v>
       </c>
-      <c r="B14" s="25" t="s">
+      <c r="B14" s="26" t="s">
         <v>62</v>
       </c>
-      <c r="C14" s="25" t="s">
+      <c r="C14" s="26" t="s">
         <v>63</v>
       </c>
-      <c r="D14" s="31" t="s">
+      <c r="D14" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="E14" s="20" t="s">
+      <c r="E14" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="F14" s="25"/>
-      <c r="G14" s="25"/>
-      <c r="H14" s="20" t="s">
+      <c r="F14" s="26"/>
+      <c r="G14" s="26"/>
+      <c r="H14" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="I14" s="25"/>
-      <c r="J14" s="25"/>
-      <c r="K14" s="25" t="s">
+      <c r="I14" s="26"/>
+      <c r="J14" s="26"/>
+      <c r="K14" s="68" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="30" t="s">
+      <c r="A15" s="29" t="s">
         <v>65</v>
       </c>
-      <c r="B15" s="25" t="s">
+      <c r="B15" s="26" t="s">
         <v>66</v>
       </c>
-      <c r="C15" s="25" t="s">
+      <c r="C15" s="26" t="s">
         <v>67</v>
       </c>
-      <c r="D15" s="31" t="s">
+      <c r="D15" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="E15" s="20" t="s">
+      <c r="E15" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="F15" s="25"/>
-      <c r="G15" s="25"/>
-      <c r="H15" s="20" t="s">
+      <c r="F15" s="26"/>
+      <c r="G15" s="26"/>
+      <c r="H15" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="I15" s="25"/>
-      <c r="J15" s="25"/>
-      <c r="K15" s="25" t="s">
+      <c r="I15" s="26"/>
+      <c r="J15" s="26"/>
+      <c r="K15" s="68" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="16" spans="1:11">
-      <c r="A16" s="30" t="s">
+      <c r="A16" s="29" t="s">
         <v>69</v>
       </c>
-      <c r="B16" s="25" t="s">
+      <c r="B16" s="26" t="s">
         <v>70</v>
       </c>
-      <c r="C16" s="25" t="s">
+      <c r="C16" s="26" t="s">
         <v>71</v>
       </c>
-      <c r="D16" s="31" t="s">
+      <c r="D16" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="E16" s="20" t="s">
+      <c r="E16" s="23" t="s">
         <v>47</v>
       </c>
-      <c r="F16" s="25"/>
-      <c r="G16" s="25"/>
-      <c r="H16" s="20" t="s">
+      <c r="F16" s="26"/>
+      <c r="G16" s="26"/>
+      <c r="H16" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="I16" s="25"/>
-      <c r="J16" s="25"/>
-      <c r="K16" s="25" t="s">
+      <c r="I16" s="26"/>
+      <c r="J16" s="26"/>
+      <c r="K16" s="68" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="17" spans="1:11">
-      <c r="A17" s="32" t="s">
+      <c r="A17" s="31" t="s">
         <v>73</v>
       </c>
-      <c r="B17" s="33" t="s">
+      <c r="B17" s="32" t="s">
         <v>74</v>
       </c>
-      <c r="C17" s="33" t="s">
+      <c r="C17" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="D17" s="34" t="s">
+      <c r="D17" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="E17" s="35" t="s">
+      <c r="E17" s="34" t="s">
         <v>76</v>
       </c>
-      <c r="F17" s="33"/>
-      <c r="G17" s="33"/>
-      <c r="H17" s="35" t="s">
+      <c r="F17" s="32"/>
+      <c r="G17" s="32"/>
+      <c r="H17" s="34" t="s">
         <v>76</v>
       </c>
-      <c r="I17" s="33"/>
-      <c r="J17" s="33"/>
-      <c r="K17" s="33" t="s">
+      <c r="I17" s="32"/>
+      <c r="J17" s="32"/>
+      <c r="K17" s="69" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="18" spans="1:11">
-      <c r="A18" s="32" t="s">
+      <c r="A18" s="31" t="s">
         <v>78</v>
       </c>
-      <c r="B18" s="33" t="s">
+      <c r="B18" s="32" t="s">
         <v>79</v>
       </c>
-      <c r="C18" s="33" t="s">
+      <c r="C18" s="32" t="s">
         <v>80</v>
       </c>
-      <c r="D18" s="34" t="s">
+      <c r="D18" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="E18" s="35" t="s">
+      <c r="E18" s="34" t="s">
         <v>76</v>
       </c>
-      <c r="F18" s="33"/>
-      <c r="G18" s="33"/>
-      <c r="H18" s="35" t="s">
+      <c r="F18" s="32"/>
+      <c r="G18" s="32"/>
+      <c r="H18" s="34" t="s">
         <v>76</v>
       </c>
-      <c r="I18" s="33"/>
-      <c r="J18" s="33"/>
-      <c r="K18" s="33" t="s">
+      <c r="I18" s="32"/>
+      <c r="J18" s="32"/>
+      <c r="K18" s="69" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="19" spans="1:11">
-      <c r="A19" s="30" t="s">
+      <c r="A19" s="29" t="s">
         <v>82</v>
       </c>
-      <c r="B19" s="25" t="s">
+      <c r="B19" s="26" t="s">
         <v>83</v>
       </c>
-      <c r="C19" s="25" t="s">
+      <c r="C19" s="26" t="s">
         <v>84</v>
       </c>
-      <c r="D19" s="31" t="s">
+      <c r="D19" s="30" t="s">
         <v>85</v>
       </c>
-      <c r="E19" s="20" t="s">
+      <c r="E19" s="23" t="s">
         <v>86</v>
       </c>
-      <c r="F19" s="20"/>
-      <c r="G19" s="20"/>
-      <c r="H19" s="20" t="s">
+      <c r="F19" s="23"/>
+      <c r="G19" s="23"/>
+      <c r="H19" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="I19" s="25"/>
-      <c r="J19" s="25"/>
-      <c r="K19" s="48" t="s">
+      <c r="I19" s="26"/>
+      <c r="J19" s="26"/>
+      <c r="K19" s="70" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="20" spans="1:11">
-      <c r="A20" s="30"/>
-      <c r="B20" s="25"/>
-      <c r="C20" s="25"/>
-      <c r="D20" s="31" t="s">
+      <c r="A20" s="29"/>
+      <c r="B20" s="26"/>
+      <c r="C20" s="26"/>
+      <c r="D20" s="30" t="s">
         <v>88</v>
       </c>
-      <c r="E20" s="20" t="s">
+      <c r="E20" s="23" t="s">
         <v>86</v>
       </c>
-      <c r="F20" s="20"/>
-      <c r="G20" s="20"/>
-      <c r="H20" s="20" t="s">
+      <c r="F20" s="23"/>
+      <c r="G20" s="23"/>
+      <c r="H20" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="I20" s="25"/>
-      <c r="J20" s="25"/>
-      <c r="K20" s="49" t="s">
+      <c r="I20" s="26"/>
+      <c r="J20" s="26"/>
+      <c r="K20" s="71" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="21" spans="1:11">
-      <c r="A21" s="30"/>
-      <c r="B21" s="25"/>
-      <c r="C21" s="25"/>
-      <c r="D21" s="31" t="s">
+      <c r="A21" s="29"/>
+      <c r="B21" s="26"/>
+      <c r="C21" s="26"/>
+      <c r="D21" s="30" t="s">
         <v>90</v>
       </c>
-      <c r="E21" s="20" t="s">
+      <c r="E21" s="23" t="s">
         <v>86</v>
       </c>
-      <c r="F21" s="20"/>
-      <c r="G21" s="20"/>
-      <c r="H21" s="20" t="s">
+      <c r="F21" s="23"/>
+      <c r="G21" s="23"/>
+      <c r="H21" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="I21" s="25"/>
-      <c r="J21" s="25"/>
-      <c r="K21" s="49" t="s">
+      <c r="I21" s="26"/>
+      <c r="J21" s="26"/>
+      <c r="K21" s="71" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="22" ht="31" customHeight="1" spans="1:11">
-      <c r="A22" s="30"/>
-      <c r="B22" s="25"/>
-      <c r="C22" s="25"/>
-      <c r="D22" s="31" t="s">
+      <c r="A22" s="29"/>
+      <c r="B22" s="26"/>
+      <c r="C22" s="26"/>
+      <c r="D22" s="30" t="s">
         <v>92</v>
       </c>
-      <c r="E22" s="20" t="s">
+      <c r="E22" s="23" t="s">
         <v>86</v>
       </c>
-      <c r="F22" s="20"/>
-      <c r="G22" s="20"/>
-      <c r="H22" s="20" t="s">
+      <c r="F22" s="23"/>
+      <c r="G22" s="23"/>
+      <c r="H22" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="I22" s="25"/>
-      <c r="J22" s="25"/>
-      <c r="K22" s="49" t="s">
+      <c r="I22" s="26"/>
+      <c r="J22" s="26"/>
+      <c r="K22" s="71" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="23" ht="62.4" spans="1:11">
-      <c r="A23" s="36" t="s">
+      <c r="A23" s="35" t="s">
         <v>94</v>
       </c>
-      <c r="B23" s="16" t="s">
+      <c r="B23" s="19" t="s">
         <v>95</v>
       </c>
-      <c r="C23" s="16" t="s">
+      <c r="C23" s="19" t="s">
         <v>96</v>
       </c>
-      <c r="D23" s="18" t="s">
+      <c r="D23" s="21" t="s">
         <v>97</v>
       </c>
-      <c r="E23" s="50" t="s">
+      <c r="E23" s="79" t="s">
         <v>98</v>
       </c>
-      <c r="F23" s="50" t="s">
+      <c r="F23" s="79" t="s">
         <v>99</v>
       </c>
-      <c r="G23" s="50" t="s">
+      <c r="G23" s="79" t="s">
         <v>100</v>
       </c>
-      <c r="H23" s="20" t="s">
+      <c r="H23" s="23" t="s">
         <v>101</v>
       </c>
-      <c r="I23" s="25"/>
-      <c r="J23" s="25"/>
-      <c r="K23" s="54" t="s">
+      <c r="I23" s="26"/>
+      <c r="J23" s="26"/>
+      <c r="K23" s="83" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="24" ht="109.2" spans="1:11">
-      <c r="A24" s="36"/>
-      <c r="B24" s="16"/>
-      <c r="C24" s="16"/>
-      <c r="D24" s="18" t="s">
+      <c r="A24" s="35"/>
+      <c r="B24" s="19"/>
+      <c r="C24" s="19"/>
+      <c r="D24" s="21" t="s">
         <v>103</v>
       </c>
-      <c r="E24" s="20" t="s">
+      <c r="E24" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="F24" s="25"/>
-      <c r="G24" s="25"/>
-      <c r="H24" s="50" t="s">
+      <c r="F24" s="26"/>
+      <c r="G24" s="26"/>
+      <c r="H24" s="79" t="s">
         <v>104</v>
       </c>
-      <c r="I24" s="19" t="s">
+      <c r="I24" s="22" t="s">
         <v>105</v>
       </c>
-      <c r="J24" s="19" t="s">
+      <c r="J24" s="22" t="s">
         <v>106</v>
       </c>
-      <c r="K24" s="47" t="s">
+      <c r="K24" s="66" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="25" ht="314" customHeight="1" spans="1:11">
-      <c r="A25" s="36" t="s">
+      <c r="A25" s="35" t="s">
         <v>108</v>
       </c>
-      <c r="B25" s="16" t="s">
+      <c r="B25" s="19" t="s">
         <v>109</v>
       </c>
-      <c r="C25" s="16" t="s">
+      <c r="C25" s="19" t="s">
         <v>110</v>
       </c>
-      <c r="D25" s="18" t="s">
+      <c r="D25" s="21" t="s">
         <v>111</v>
       </c>
-      <c r="E25" s="20" t="s">
+      <c r="E25" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="F25" s="25"/>
-      <c r="G25" s="25"/>
-      <c r="H25" s="50" t="s">
+      <c r="F25" s="26"/>
+      <c r="G25" s="26"/>
+      <c r="H25" s="79" t="s">
         <v>112</v>
       </c>
-      <c r="I25" s="19" t="s">
+      <c r="I25" s="22" t="s">
         <v>113</v>
       </c>
-      <c r="J25" s="55" t="s">
+      <c r="J25" s="84" t="s">
         <v>114</v>
       </c>
-      <c r="K25" s="47" t="s">
+      <c r="K25" s="66" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="26" ht="163" customHeight="1" spans="1:11">
-      <c r="A26" s="36"/>
-      <c r="B26" s="16"/>
-      <c r="C26" s="16"/>
-      <c r="D26" s="18" t="s">
+      <c r="A26" s="35"/>
+      <c r="B26" s="19"/>
+      <c r="C26" s="19"/>
+      <c r="D26" s="21" t="s">
         <v>116</v>
       </c>
-      <c r="E26" s="20" t="s">
+      <c r="E26" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="F26" s="25"/>
-      <c r="G26" s="25"/>
-      <c r="H26" s="50" t="s">
+      <c r="F26" s="26"/>
+      <c r="G26" s="26"/>
+      <c r="H26" s="79" t="s">
         <v>117</v>
       </c>
-      <c r="I26" s="19" t="s">
+      <c r="I26" s="22" t="s">
         <v>118</v>
       </c>
-      <c r="J26" s="55" t="s">
+      <c r="J26" s="84" t="s">
         <v>119</v>
       </c>
-      <c r="K26" s="47" t="s">
+      <c r="K26" s="66" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="27" ht="126" customHeight="1" spans="1:11">
-      <c r="A27" s="36" t="s">
+      <c r="A27" s="35" t="s">
         <v>121</v>
       </c>
       <c r="B27" s="36" t="s">
@@ -2987,193 +3650,563 @@
       <c r="C27" s="36" t="s">
         <v>123</v>
       </c>
-      <c r="D27" s="18" t="s">
+      <c r="D27" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="E27" s="56" t="s">
+      <c r="E27" s="85" t="s">
         <v>124</v>
       </c>
-      <c r="F27" s="19" t="s">
+      <c r="F27" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="G27" s="55" t="s">
+      <c r="G27" s="84" t="s">
         <v>125</v>
       </c>
-      <c r="H27" s="20" t="s">
+      <c r="H27" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="I27" s="25"/>
-      <c r="J27" s="25"/>
-      <c r="K27" s="30" t="s">
+      <c r="I27" s="26"/>
+      <c r="J27" s="26"/>
+      <c r="K27" s="72" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="28" spans="1:11">
-      <c r="A28" s="36" t="s">
+      <c r="A28" s="38" t="s">
         <v>127</v>
       </c>
-      <c r="B28" s="16" t="s">
+      <c r="B28" s="39" t="s">
         <v>128</v>
       </c>
-      <c r="C28" s="16" t="s">
+      <c r="C28" s="39" t="s">
         <v>129</v>
       </c>
-      <c r="D28" s="18" t="s">
+      <c r="D28" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="E28" s="35" t="s">
+      <c r="E28" s="41" t="s">
         <v>130</v>
       </c>
-      <c r="F28" s="35"/>
-      <c r="G28" s="35"/>
-      <c r="H28" s="20" t="s">
+      <c r="F28" s="41"/>
+      <c r="G28" s="41"/>
+      <c r="H28" s="41" t="s">
         <v>19</v>
       </c>
-      <c r="I28" s="25"/>
-      <c r="J28" s="25"/>
-      <c r="K28" s="51" t="s">
+      <c r="I28" s="41"/>
+      <c r="J28" s="41"/>
+      <c r="K28" s="65"/>
+    </row>
+    <row r="29" ht="96" customHeight="1" spans="1:11">
+      <c r="A29" s="42" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="29" ht="96" customHeight="1" spans="1:11">
-      <c r="A29" s="38" t="s">
+      <c r="B29" s="25" t="s">
         <v>132</v>
       </c>
-      <c r="B29" s="22" t="s">
+      <c r="C29" s="25" t="s">
         <v>133</v>
       </c>
-      <c r="C29" s="22" t="s">
+      <c r="D29" s="21" t="s">
+        <v>15</v>
+      </c>
+      <c r="E29" s="86" t="s">
         <v>134</v>
       </c>
-      <c r="D29" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="E29" s="57" t="s">
+      <c r="F29" s="44" t="s">
+        <v>17</v>
+      </c>
+      <c r="G29" s="44" t="s">
         <v>135</v>
       </c>
-      <c r="F29" s="40" t="s">
-        <v>17</v>
-      </c>
-      <c r="G29" s="40" t="s">
+      <c r="H29" s="23" t="s">
+        <v>19</v>
+      </c>
+      <c r="I29" s="26"/>
+      <c r="J29" s="26"/>
+      <c r="K29" s="66" t="s">
         <v>136</v>
       </c>
-      <c r="H29" s="20" t="s">
+    </row>
+    <row r="30" ht="258.6" customHeight="1" spans="1:11">
+      <c r="A30" s="42"/>
+      <c r="B30" s="25"/>
+      <c r="C30" s="25"/>
+      <c r="D30" s="21" t="s">
+        <v>137</v>
+      </c>
+      <c r="E30" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="I29" s="25"/>
-      <c r="J29" s="25"/>
-      <c r="K29" s="47" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="30" ht="258.6" customHeight="1" spans="1:11">
-      <c r="A30" s="41"/>
-      <c r="B30" s="24"/>
-      <c r="C30" s="24"/>
-      <c r="D30" s="18" t="s">
+      <c r="F30" s="26"/>
+      <c r="G30" s="26"/>
+      <c r="H30" s="79" t="s">
         <v>138</v>
       </c>
-      <c r="E30" s="20" t="s">
-        <v>19</v>
-      </c>
-      <c r="F30" s="25"/>
-      <c r="G30" s="25"/>
-      <c r="H30" s="50" t="s">
+      <c r="I30" s="22" t="s">
         <v>139</v>
       </c>
-      <c r="I30" s="19" t="s">
+      <c r="J30" s="79" t="s">
         <v>140</v>
       </c>
-      <c r="J30" s="50" t="s">
+      <c r="K30" s="66" t="s">
         <v>141</v>
-      </c>
-      <c r="K30" s="47" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="31" ht="141" customHeight="1" spans="1:11">
       <c r="A31" s="42"/>
-      <c r="B31" s="29"/>
-      <c r="C31" s="29"/>
-      <c r="D31" s="18" t="s">
+      <c r="B31" s="25"/>
+      <c r="C31" s="25"/>
+      <c r="D31" s="21" t="s">
+        <v>142</v>
+      </c>
+      <c r="E31" s="23"/>
+      <c r="F31" s="26"/>
+      <c r="G31" s="26"/>
+      <c r="H31" s="79" t="s">
         <v>143</v>
       </c>
-      <c r="E31" s="20"/>
-      <c r="F31" s="25"/>
-      <c r="G31" s="25"/>
-      <c r="H31" s="50" t="s">
+      <c r="I31" s="22" t="s">
         <v>144</v>
       </c>
-      <c r="I31" s="19" t="s">
+      <c r="J31" s="22" t="s">
+        <v>135</v>
+      </c>
+      <c r="K31" s="66" t="s">
         <v>145</v>
       </c>
-      <c r="J31" s="19" t="s">
-        <v>136</v>
-      </c>
-      <c r="K31" s="47" t="s">
+    </row>
+    <row r="32" spans="1:11">
+      <c r="A32" s="35" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="32" spans="1:11">
-      <c r="A32" s="36" t="s">
+      <c r="B32" s="19" t="s">
         <v>147</v>
       </c>
-      <c r="B32" s="16" t="s">
+      <c r="C32" s="19" t="s">
         <v>148</v>
       </c>
-      <c r="C32" s="16" t="s">
+      <c r="D32" s="21" t="s">
+        <v>15</v>
+      </c>
+      <c r="E32" s="23" t="s">
         <v>149</v>
       </c>
-      <c r="D32" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="E32" s="20" t="s">
+      <c r="F32" s="26"/>
+      <c r="G32" s="26"/>
+      <c r="H32" s="23" t="s">
+        <v>19</v>
+      </c>
+      <c r="I32" s="26"/>
+      <c r="J32" s="26"/>
+      <c r="K32" s="65" t="s">
         <v>150</v>
       </c>
-      <c r="F32" s="25"/>
-      <c r="G32" s="25"/>
-      <c r="H32" s="20" t="s">
+    </row>
+    <row r="33" ht="46.8" spans="1:11">
+      <c r="A33" s="35" t="s">
+        <v>151</v>
+      </c>
+      <c r="B33" s="19" t="s">
+        <v>152</v>
+      </c>
+      <c r="C33" s="19" t="s">
+        <v>153</v>
+      </c>
+      <c r="D33" s="21" t="s">
+        <v>154</v>
+      </c>
+      <c r="E33" s="45" t="s">
+        <v>155</v>
+      </c>
+      <c r="F33" s="46" t="s">
+        <v>156</v>
+      </c>
+      <c r="G33" s="46" t="s">
+        <v>157</v>
+      </c>
+      <c r="H33" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="I32" s="25"/>
-      <c r="J32" s="25"/>
-      <c r="K32" s="16" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="33" ht="46.8" spans="1:11">
-      <c r="A33" s="36" t="s">
-        <v>152</v>
-      </c>
-      <c r="B33" s="16" t="s">
-        <v>153</v>
-      </c>
-      <c r="C33" s="16" t="s">
-        <v>154</v>
-      </c>
-      <c r="D33" s="18" t="s">
-        <v>155</v>
-      </c>
-      <c r="E33" s="43" t="s">
-        <v>156</v>
-      </c>
-      <c r="F33" s="44" t="s">
-        <v>157</v>
-      </c>
-      <c r="G33" s="44" t="s">
+      <c r="I33" s="26"/>
+      <c r="J33" s="26"/>
+      <c r="K33" s="65" t="s">
         <v>158</v>
       </c>
-      <c r="H33" s="20" t="s">
+    </row>
+    <row r="34" spans="1:11">
+      <c r="A34" s="47" t="s">
+        <v>159</v>
+      </c>
+      <c r="B34" s="48" t="s">
+        <v>160</v>
+      </c>
+      <c r="C34" s="48" t="s">
+        <v>161</v>
+      </c>
+      <c r="D34" s="49" t="s">
+        <v>162</v>
+      </c>
+      <c r="E34" s="48" t="s">
+        <v>163</v>
+      </c>
+      <c r="F34" s="48"/>
+      <c r="G34" s="48"/>
+      <c r="H34" s="48"/>
+      <c r="I34" s="48"/>
+      <c r="J34" s="48"/>
+      <c r="K34" s="73"/>
+    </row>
+    <row r="35" ht="31.2" spans="1:11">
+      <c r="A35" s="50" t="s">
+        <v>164</v>
+      </c>
+      <c r="B35" s="48" t="s">
+        <v>165</v>
+      </c>
+      <c r="C35" s="48" t="s">
+        <v>166</v>
+      </c>
+      <c r="D35" s="49" t="s">
+        <v>162</v>
+      </c>
+      <c r="E35" s="48" t="s">
+        <v>163</v>
+      </c>
+      <c r="F35" s="48"/>
+      <c r="G35" s="48"/>
+      <c r="H35" s="48"/>
+      <c r="I35" s="48"/>
+      <c r="J35" s="48"/>
+      <c r="K35" s="73"/>
+    </row>
+    <row r="36" ht="31.2" spans="1:11">
+      <c r="A36" s="51" t="s">
+        <v>167</v>
+      </c>
+      <c r="B36" s="52" t="s">
+        <v>168</v>
+      </c>
+      <c r="C36" s="52" t="s">
+        <v>169</v>
+      </c>
+      <c r="D36" s="53" t="s">
+        <v>170</v>
+      </c>
+      <c r="E36" s="54" t="s">
+        <v>171</v>
+      </c>
+      <c r="F36" s="87" t="s">
+        <v>172</v>
+      </c>
+      <c r="G36" s="52" t="s">
+        <v>173</v>
+      </c>
+      <c r="H36" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="I33" s="25"/>
-      <c r="J33" s="25"/>
-      <c r="K33" s="16" t="s">
-        <v>159</v>
+      <c r="I36" s="26"/>
+      <c r="J36" s="26"/>
+      <c r="K36" s="74" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="37" ht="93.6" spans="1:11">
+      <c r="A37" s="51"/>
+      <c r="B37" s="52"/>
+      <c r="C37" s="52"/>
+      <c r="D37" s="55" t="s">
+        <v>175</v>
+      </c>
+      <c r="E37" s="23" t="s">
+        <v>19</v>
+      </c>
+      <c r="F37" s="26"/>
+      <c r="G37" s="26"/>
+      <c r="H37" s="52" t="s">
+        <v>176</v>
+      </c>
+      <c r="I37" s="22" t="s">
+        <v>177</v>
+      </c>
+      <c r="J37" s="52" t="s">
+        <v>178</v>
+      </c>
+      <c r="K37" s="75" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="38" ht="31.2" spans="1:11">
+      <c r="A38" s="51"/>
+      <c r="B38" s="52"/>
+      <c r="C38" s="52"/>
+      <c r="D38" s="53" t="s">
+        <v>180</v>
+      </c>
+      <c r="E38" s="23" t="s">
+        <v>19</v>
+      </c>
+      <c r="F38" s="26"/>
+      <c r="G38" s="26"/>
+      <c r="H38" s="54" t="s">
+        <v>181</v>
+      </c>
+      <c r="I38" s="87" t="s">
+        <v>172</v>
+      </c>
+      <c r="J38" s="52" t="s">
+        <v>173</v>
+      </c>
+      <c r="K38" s="75" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="39" ht="109.2" spans="1:11">
+      <c r="A39" s="51" t="s">
+        <v>183</v>
+      </c>
+      <c r="B39" s="52" t="s">
+        <v>184</v>
+      </c>
+      <c r="C39" s="52" t="s">
+        <v>185</v>
+      </c>
+      <c r="D39" s="53" t="s">
+        <v>186</v>
+      </c>
+      <c r="E39" s="23" t="s">
+        <v>19</v>
+      </c>
+      <c r="F39" s="26"/>
+      <c r="G39" s="26"/>
+      <c r="H39" s="54" t="s">
+        <v>187</v>
+      </c>
+      <c r="I39" s="76" t="s">
+        <v>188</v>
+      </c>
+      <c r="J39" s="54" t="s">
+        <v>189</v>
+      </c>
+      <c r="K39" s="75" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="40" ht="280.8" spans="1:11">
+      <c r="A40" s="51"/>
+      <c r="B40" s="52"/>
+      <c r="C40" s="52"/>
+      <c r="D40" s="53" t="s">
+        <v>191</v>
+      </c>
+      <c r="E40" s="52" t="s">
+        <v>192</v>
+      </c>
+      <c r="F40" s="54" t="s">
+        <v>193</v>
+      </c>
+      <c r="G40" s="56" t="s">
+        <v>194</v>
+      </c>
+      <c r="H40" s="23" t="s">
+        <v>19</v>
+      </c>
+      <c r="I40" s="26"/>
+      <c r="J40" s="26"/>
+      <c r="K40" s="77" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="41" ht="374.4" spans="1:11">
+      <c r="A41" s="51"/>
+      <c r="B41" s="52"/>
+      <c r="C41" s="52"/>
+      <c r="D41" s="53" t="s">
+        <v>196</v>
+      </c>
+      <c r="E41" s="54" t="s">
+        <v>197</v>
+      </c>
+      <c r="F41" s="54" t="s">
+        <v>193</v>
+      </c>
+      <c r="G41" s="56" t="s">
+        <v>198</v>
+      </c>
+      <c r="H41" s="23" t="s">
+        <v>19</v>
+      </c>
+      <c r="I41" s="26"/>
+      <c r="J41" s="26"/>
+      <c r="K41" s="77" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="42" ht="78" spans="1:11">
+      <c r="A42" s="51"/>
+      <c r="B42" s="52"/>
+      <c r="C42" s="52"/>
+      <c r="D42" s="53" t="s">
+        <v>199</v>
+      </c>
+      <c r="E42" s="23" t="s">
+        <v>19</v>
+      </c>
+      <c r="F42" s="26"/>
+      <c r="G42" s="26"/>
+      <c r="H42" s="54" t="s">
+        <v>200</v>
+      </c>
+      <c r="I42" s="52" t="s">
+        <v>201</v>
+      </c>
+      <c r="J42" s="54" t="s">
+        <v>202</v>
+      </c>
+      <c r="K42" s="75" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="43" ht="109.2" spans="1:11">
+      <c r="A43" s="51" t="s">
+        <v>204</v>
+      </c>
+      <c r="B43" s="52" t="s">
+        <v>205</v>
+      </c>
+      <c r="C43" s="52" t="s">
+        <v>206</v>
+      </c>
+      <c r="D43" s="53" t="s">
+        <v>207</v>
+      </c>
+      <c r="E43" s="52" t="s">
+        <v>208</v>
+      </c>
+      <c r="F43" s="57" t="s">
+        <v>165</v>
+      </c>
+      <c r="G43" s="54" t="s">
+        <v>209</v>
+      </c>
+      <c r="H43" s="23" t="s">
+        <v>19</v>
+      </c>
+      <c r="I43" s="26"/>
+      <c r="J43" s="26"/>
+      <c r="K43" s="75" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="44" ht="218.4" spans="1:11">
+      <c r="A44" s="51"/>
+      <c r="B44" s="52"/>
+      <c r="C44" s="52"/>
+      <c r="D44" s="53" t="s">
+        <v>211</v>
+      </c>
+      <c r="E44" s="52" t="s">
+        <v>212</v>
+      </c>
+      <c r="F44" s="57" t="s">
+        <v>165</v>
+      </c>
+      <c r="G44" s="54" t="s">
+        <v>213</v>
+      </c>
+      <c r="H44" s="52" t="s">
+        <v>214</v>
+      </c>
+      <c r="I44" s="54" t="s">
+        <v>215</v>
+      </c>
+      <c r="J44" s="52" t="s">
+        <v>216</v>
+      </c>
+      <c r="K44" s="75" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="45" ht="124.8" spans="1:11">
+      <c r="A45" s="51"/>
+      <c r="B45" s="52"/>
+      <c r="C45" s="52"/>
+      <c r="D45" s="53" t="s">
+        <v>218</v>
+      </c>
+      <c r="E45" s="52" t="s">
+        <v>219</v>
+      </c>
+      <c r="F45" s="57" t="s">
+        <v>165</v>
+      </c>
+      <c r="G45" s="54" t="s">
+        <v>220</v>
+      </c>
+      <c r="H45" s="23" t="s">
+        <v>19</v>
+      </c>
+      <c r="I45" s="26"/>
+      <c r="J45" s="26"/>
+      <c r="K45" s="75" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="46" ht="124.8" spans="1:11">
+      <c r="A46" s="51"/>
+      <c r="B46" s="52"/>
+      <c r="C46" s="52"/>
+      <c r="D46" s="53" t="s">
+        <v>222</v>
+      </c>
+      <c r="E46" s="52" t="s">
+        <v>223</v>
+      </c>
+      <c r="F46" s="57" t="s">
+        <v>165</v>
+      </c>
+      <c r="G46" s="54" t="s">
+        <v>224</v>
+      </c>
+      <c r="H46" s="23" t="s">
+        <v>19</v>
+      </c>
+      <c r="I46" s="26"/>
+      <c r="J46" s="26"/>
+      <c r="K46" s="75" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="47" ht="328.35" spans="1:11">
+      <c r="A47" s="58"/>
+      <c r="B47" s="59"/>
+      <c r="C47" s="59"/>
+      <c r="D47" s="60" t="s">
+        <v>226</v>
+      </c>
+      <c r="E47" s="59" t="s">
+        <v>227</v>
+      </c>
+      <c r="F47" s="61" t="s">
+        <v>165</v>
+      </c>
+      <c r="G47" s="62" t="s">
+        <v>228</v>
+      </c>
+      <c r="H47" s="59" t="s">
+        <v>229</v>
+      </c>
+      <c r="I47" s="62" t="s">
+        <v>230</v>
+      </c>
+      <c r="J47" s="59" t="s">
+        <v>231</v>
+      </c>
+      <c r="K47" s="78" t="s">
+        <v>232</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="65">
+  <mergeCells count="84">
     <mergeCell ref="E2:G2"/>
     <mergeCell ref="H2:J2"/>
     <mergeCell ref="H4:J4"/>
@@ -3212,31 +4245,50 @@
     <mergeCell ref="E25:G25"/>
     <mergeCell ref="E26:G26"/>
     <mergeCell ref="H27:J27"/>
-    <mergeCell ref="E28:G28"/>
-    <mergeCell ref="H28:J28"/>
     <mergeCell ref="H29:J29"/>
     <mergeCell ref="E30:G30"/>
     <mergeCell ref="E32:G32"/>
     <mergeCell ref="H32:J32"/>
     <mergeCell ref="H33:J33"/>
+    <mergeCell ref="E34:K34"/>
+    <mergeCell ref="E35:K35"/>
+    <mergeCell ref="H36:J36"/>
+    <mergeCell ref="E37:G37"/>
+    <mergeCell ref="E38:G38"/>
+    <mergeCell ref="E39:G39"/>
+    <mergeCell ref="H40:J40"/>
+    <mergeCell ref="H41:J41"/>
+    <mergeCell ref="E42:G42"/>
+    <mergeCell ref="H43:J43"/>
+    <mergeCell ref="H45:J45"/>
+    <mergeCell ref="H46:J46"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="A5:A9"/>
     <mergeCell ref="A19:A22"/>
     <mergeCell ref="A23:A24"/>
     <mergeCell ref="A25:A26"/>
     <mergeCell ref="A29:A31"/>
+    <mergeCell ref="A36:A38"/>
+    <mergeCell ref="A39:A42"/>
+    <mergeCell ref="A43:A47"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="B5:B9"/>
     <mergeCell ref="B19:B22"/>
     <mergeCell ref="B23:B24"/>
     <mergeCell ref="B25:B26"/>
     <mergeCell ref="B29:B31"/>
+    <mergeCell ref="B36:B38"/>
+    <mergeCell ref="B39:B42"/>
+    <mergeCell ref="B43:B47"/>
     <mergeCell ref="C2:C3"/>
     <mergeCell ref="C5:C9"/>
     <mergeCell ref="C19:C22"/>
     <mergeCell ref="C23:C24"/>
     <mergeCell ref="C25:C26"/>
     <mergeCell ref="C29:C31"/>
+    <mergeCell ref="C36:C38"/>
+    <mergeCell ref="C39:C42"/>
+    <mergeCell ref="C43:C47"/>
     <mergeCell ref="D2:D3"/>
     <mergeCell ref="K2:K3"/>
   </mergeCells>

</xml_diff>